<commit_message>
feat: allow admins to delete papers and notes
</commit_message>
<xml_diff>
--- a/OurBUT_需求整理文档.xlsx
+++ b/OurBUT_需求整理文档.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet name="需求总览" sheetId="1" r:id="rId1"/>
     <sheet name="逻辑规则详解" sheetId="2" r:id="rId2"/>
-    <sheet name="待确认问题清单" sheetId="3" r:id="rId3"/>
-    <sheet name="修改点" sheetId="4" r:id="rId4"/>
+    <sheet name="已确认问题清单" sheetId="3" r:id="rId3"/>
+    <sheet name="4月5日修改点" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="176">
   <si>
     <t>OurBUT 产品需求总览（按模块整理）</t>
   </si>
@@ -343,12 +343,185 @@
     <t>系统每周日23:59自动执行</t>
   </si>
   <si>
-    <t>1. 判断条件：注册用户连续两个自然周评论次数均为0
-2. 新注册用户前两周设置免检观察期
-3. 请假已通过的周不计入连续0评论
-4. 停用动作：账号status改为inactive，无法登录
-5. 通知：老师账号消息中心推送，含姓名+停用时间
-6. 恢复：管理员后台手动重新激活，用户收到通知</t>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>判断条件：注册用户连续两个自然周评论次数均为</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">0
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>新注册用户前两周设置免检观察期</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>请假已通过的周不计入连续</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>评论</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+4. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>停用动作：账号</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>改为</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>inactive</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>，无法登录</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+5. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>通知：老师账号消息中心推送，含姓名</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>停用时间</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+6. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>恢复：管理员后台手动重新激活，用户收到通知</t>
+    </r>
   </si>
   <si>
     <t>账号停用后历史数据是否保留？可以恢复还是永久注销？老师消息中心入口是否已有？可保留，需新增全员的消息中心入口。（历史数据保留，可以恢复，在个人页新增消息中心）</t>
@@ -2002,43 +2175,7 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>停用动作：账号</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>status</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>改为</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>inactive</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>，无法登录</t>
+      <t>停用动作：需管理员手动停用</t>
     </r>
     <r>
       <rPr>
@@ -2057,25 +2194,7 @@
         <rFont val="宋体-简"/>
         <charset val="134"/>
       </rPr>
-      <t>通知：老师账号消息中心推送，含姓名</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>+</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>停用时间</t>
+      <t>通知：老师账号消息中心推送</t>
     </r>
     <r>
       <rPr>
@@ -3334,172 +3453,172 @@
     <t>建议上限3条，显示金色「精选」徽章</t>
   </si>
   <si>
+    <t>账号停用后数据是否全量保留？能否恢复登录？</t>
+  </si>
+  <si>
+    <t>建议保留，管理员可一键恢复。硬删除不可逆，不建议</t>
+  </si>
+  <si>
+    <t>新注册用户前两周是否设置免检观察期？</t>
+  </si>
+  <si>
+    <t>建议设置2周免检期，避免新人被误停用</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>改成</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>周免检期</t>
+    </r>
+  </si>
+  <si>
+    <t>请假仅作备案还是会影响出勤统计？该功能实际使用价值有多大？</t>
+  </si>
+  <si>
+    <t>建议先做最轻量版（提交+老师收到通知），出勤统计后续看需求再加</t>
+  </si>
+  <si>
+    <t>需要增加出勤统计，逻辑规则已写</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>名片卡的入口在哪里？是否支持搜索/筛选全员名单？</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>建议三个入口均支持：任务与出勤头像点击、评论区作者名、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>BUT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>成员页</t>
+    </r>
+  </si>
+  <si>
+    <t>个人收藏是否区分「文献」和「评论/idea」两种类型？</t>
+  </si>
+  <si>
+    <t>建议区分，分两个子tab展示</t>
+  </si>
+  <si>
+    <t>历史数据统计移走后放在个人主页的哪个位置？</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>建议个人主页新增「我的贡献」卡片，含上传数</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>评论数</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
+      <t>完成率</t>
+    </r>
+  </si>
+  <si>
+    <t>数据迁移的停机时间窗口如何安排？是否需要提前公告用户？</t>
+  </si>
+  <si>
+    <t>建议选周日凌晨2-4点，公告提前3天发出</t>
+  </si>
+  <si>
+    <t>暂不做</t>
+  </si>
+  <si>
+    <t>邮箱验证是否强制？还是可选（先注册后验证）？</t>
+  </si>
+  <si>
+    <t>建议强制，未验证账号只读，引导完成验证后解锁功能</t>
+  </si>
+  <si>
+    <t>未验证帐号不可登陆</t>
+  </si>
+  <si>
     <t>本科生S&amp;N板块的期刊号分类格式如何定义？</t>
   </si>
   <si>
     <t>建议老师提供统一规则，开发按规则硬编码下拉选项</t>
-  </si>
-  <si>
-    <t>暂不做</t>
-  </si>
-  <si>
-    <t>账号停用后数据是否全量保留？能否恢复登录？</t>
-  </si>
-  <si>
-    <t>建议保留，管理员可一键恢复。硬删除不可逆，不建议</t>
-  </si>
-  <si>
-    <t>新注册用户前两周是否设置免检观察期？</t>
-  </si>
-  <si>
-    <t>建议设置2周免检期，避免新人被误停用</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFC00000"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>改成</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color rgb="FFC00000"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>周免检期</t>
-    </r>
-  </si>
-  <si>
-    <t>邮箱验证是否强制？还是可选（先注册后验证）？</t>
-  </si>
-  <si>
-    <t>建议强制，未验证账号只读，引导完成验证后解锁功能</t>
-  </si>
-  <si>
-    <t>未验证帐号不可登陆</t>
-  </si>
-  <si>
-    <t>请假仅作备案还是会影响出勤统计？该功能实际使用价值有多大？</t>
-  </si>
-  <si>
-    <t>建议先做最轻量版（提交+老师收到通知），出勤统计后续看需求再加</t>
-  </si>
-  <si>
-    <t>需要增加出勤统计，逻辑规则已写</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>名片卡的入口在哪里？是否支持搜索/筛选全员名单？</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>建议三个入口均支持：任务与出勤头像点击、评论区作者名、</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>BUT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>成员页</t>
-    </r>
-  </si>
-  <si>
-    <t>个人收藏是否区分「文献」和「评论/idea」两种类型？</t>
-  </si>
-  <si>
-    <t>建议区分，分两个子tab展示</t>
-  </si>
-  <si>
-    <t>历史数据统计移走后放在个人主页的哪个位置？</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>建议个人主页新增「我的贡献」卡片，含上传数</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>评论数</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF595959"/>
-        <rFont val="宋体-简"/>
-        <charset val="134"/>
-      </rPr>
-      <t>完成率</t>
-    </r>
-  </si>
-  <si>
-    <t>数据迁移的停机时间窗口如何安排？是否需要提前公告用户？</t>
-  </si>
-  <si>
-    <t>建议选周日凌晨2-4点，公告提前3天发出</t>
   </si>
   <si>
     <t>修改点</t>
@@ -3548,13 +3667,21 @@
 2、消息显示后，需要点击可查看具体信息内容，给一个弹窗查看消息，消息需要有年月日时间，需要有消息分类，请假消息、审批消息、退出组织消息三类。
 3、请假消息：就是管理员收到同学请假申请后，就出现在这一类，然后弹窗内，有请假审批按钮，点击即为审批通过，也可以点击驳回。
 4、审批消息：同学请假申请通过后，会返回给同学请假审批已通过的消息。
-5、退出组织消息：为连续两周评论数为0的同学，提醒已自动停用帐号，若有特殊情况请联系老师沟通。</t>
+5、退出组织消息：为连续两周评论数为0的同学，提醒同学即将停用帐号，若有特殊情况请联系老师沟通。管理员手动停用帐号。</t>
+  </si>
+  <si>
+    <t>笔记板块</t>
+  </si>
+  <si>
+    <t>1、新增笔记上传板块：包括笔记标题、笔记时间、笔记该要，笔记可上传pdf或者9张jpg格式
+2、个人资料新增我的笔记板块，可以阅读和删除
+3、成员卡片可以阅读我的笔记，隐藏我的收藏。</t>
   </si>
   <si>
     <t>模拟数据</t>
   </si>
   <si>
-    <t>帮我输入一套数据，做模拟数据展示，比如成员多生成几个，评论，还有请假数据，点赞等</t>
+    <t>本地造数据，做模拟数据展示，比如成员多生成几个，评论，还有请假数据，点赞等</t>
   </si>
 </sst>
 </file>
@@ -3805,7 +3932,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="42">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3832,7 +3959,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE2E2"/>
+        <fgColor theme="0" tint="-0.15"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3844,13 +3977,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
+        <fgColor rgb="FFFFE2E2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3863,6 +3990,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5F5F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4192,7 +4325,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -4216,7 +4349,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
@@ -4225,7 +4358,7 @@
     <xf numFmtId="0" fontId="22" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -4234,89 +4367,89 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4339,70 +4472,88 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -4796,344 +4947,344 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" ht="72" customHeight="1" spans="1:8">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="G4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="31" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" ht="72" customHeight="1" spans="1:8">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="27" t="s">
+      <c r="H5" s="31" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" ht="72" customHeight="1" spans="1:8">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="25" t="s">
+      <c r="F6" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="27" t="s">
+      <c r="H6" s="31" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" ht="72" customHeight="1" spans="1:8">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="25" t="s">
+      <c r="G7" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="H7" s="27" t="s">
+      <c r="H7" s="33" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:1">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1" spans="1:8">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="25" t="s">
+      <c r="F9" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="25" t="s">
+      <c r="G9" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="H9" s="27" t="s">
+      <c r="H9" s="31" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="10" ht="72" customHeight="1" spans="1:8">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="34" t="s">
         <v>45</v>
       </c>
-      <c r="H10" s="27" t="s">
+      <c r="H10" s="33" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:1">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="12" ht="72" customHeight="1" spans="1:8">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F12" s="25" t="s">
+      <c r="F12" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="G12" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="27" t="s">
+      <c r="H12" s="31" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1" spans="1:8">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="E13" s="29" t="s">
+      <c r="E13" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="29" t="s">
+      <c r="F13" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G13" s="29" t="s">
+      <c r="G13" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="H13" s="27" t="s">
+      <c r="H13" s="31" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" ht="72" customHeight="1" spans="1:8">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="C14" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="29" t="s">
+      <c r="E14" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="29" t="s">
+      <c r="F14" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="29" t="s">
+      <c r="G14" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="H14" s="27" t="s">
+      <c r="H14" s="31" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:1">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="16" ht="72" customHeight="1" spans="1:8">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="D16" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E16" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="29" t="s">
+      <c r="F16" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G16" s="29" t="s">
+      <c r="G16" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="H16" s="27" t="s">
+      <c r="H16" s="31" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:1">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="16" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="18" ht="72" customHeight="1" spans="1:8">
-      <c r="A18" s="24" t="s">
+      <c r="A18" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="B18" s="24" t="s">
+      <c r="B18" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="E18" s="29" t="s">
+      <c r="E18" s="35" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="G18" s="29" t="s">
+      <c r="G18" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="H18" s="27" t="s">
+      <c r="H18" s="33" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:1">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="16" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="20" ht="72" customHeight="1" spans="1:8">
-      <c r="A20" s="23" t="s">
+      <c r="A20" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="D20" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="E20" s="28" t="s">
+      <c r="E20" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="F20" s="28" t="s">
+      <c r="F20" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="G20" s="28" t="s">
+      <c r="G20" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="H20" s="27" t="s">
+      <c r="H20" s="33" t="s">
         <v>85</v>
       </c>
     </row>
@@ -5184,200 +5335,200 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:1">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" ht="88" customHeight="1" spans="1:4">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="17" t="s">
         <v>90</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="19" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="5" ht="88" customHeight="1" spans="1:4">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>93</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="19" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="6" ht="88" customHeight="1" spans="1:4">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>96</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="19" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="7" ht="88" customHeight="1" spans="1:4">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="22" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:1">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="9" ht="88" customHeight="1" spans="1:4">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="17" t="s">
         <v>102</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="10" ht="88" customHeight="1" spans="1:4">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="23" t="s">
         <v>105</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="22" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:1">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="12" ht="88" customHeight="1" spans="1:4">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="17" t="s">
         <v>108</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="19" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="13" ht="88" customHeight="1" spans="1:4">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="19" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="14" ht="88" customHeight="1" spans="1:4">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="19" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:1">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="16" ht="88" customHeight="1" spans="1:4">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D16" s="19" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:1">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="16" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="18" ht="88" customHeight="1" spans="1:4">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="22" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:1">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="16" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="20" ht="88" customHeight="1" spans="1:4">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="23" t="s">
         <v>123</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="22" t="s">
         <v>125</v>
       </c>
     </row>
@@ -5448,10 +5599,10 @@
       <c r="D3" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="14" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5468,10 +5619,10 @@
       <c r="D4" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="14" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5488,10 +5639,10 @@
       <c r="D5" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="14" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5500,19 +5651,19 @@
         <v>29</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="F6" s="13" t="s">
-        <v>140</v>
+      <c r="F6" s="14" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1" spans="1:6">
@@ -5526,13 +5677,13 @@
         <v>12</v>
       </c>
       <c r="D7" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="F7" s="14" t="s">
         <v>142</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1" spans="1:6">
@@ -5540,7 +5691,7 @@
         <v>42</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>12</v>
@@ -5548,10 +5699,10 @@
       <c r="D8" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="14" t="s">
         <v>145</v>
       </c>
     </row>
@@ -5559,20 +5710,20 @@
       <c r="A9" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>30</v>
+      <c r="B9" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>146</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="E9" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="E9" s="15" t="s">
         <v>148</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1" spans="1:6">
@@ -5583,35 +5734,35 @@
         <v>49</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>12</v>
+        <v>146</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="F10" s="13" t="s">
-        <v>151</v>
+      <c r="F10" s="14" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1" spans="1:6">
       <c r="A11" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="11" t="s">
+      <c r="B11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="E11" s="15" t="s">
         <v>152</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="14" t="s">
         <v>133</v>
       </c>
     </row>
@@ -5619,60 +5770,60 @@
       <c r="A12" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="B12" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>155</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1" spans="1:6">
       <c r="A13" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="9" t="s">
+      <c r="B13" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="E13" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="F13" s="14" t="s">
         <v>158</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1" spans="1:6">
       <c r="A14" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="B14" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="F14" s="13" t="s">
-        <v>140</v>
+      <c r="F14" s="14" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -5687,8 +5838,8 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="3"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="7" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="2" width="37.6538461538462" style="1" customWidth="1"/>
     <col min="3" max="3" width="88.625" style="1" customWidth="1"/>
@@ -5765,15 +5916,26 @@
         <v>171</v>
       </c>
     </row>
-    <row r="7" ht="77" customHeight="1" spans="1:3">
+    <row r="7" ht="130" customHeight="1" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>172</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="4" t="s">
         <v>173</v>
+      </c>
+    </row>
+    <row r="8" ht="77" customHeight="1" spans="1:3">
+      <c r="A8" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>